<commit_message>
update cliping models and start simulation script
1. add print statement to know when the script finished to clip the models
2. Add print statement when the clipping script is clipping rasters.
3. Update simulations_id excel file. Add more columns.
4. update Start simulation to make sure the initial water levels 1d and 2d are set.
</commit_message>
<xml_diff>
--- a/hhnk_threedi_tools/breaches/start_download_simulation/simulations_id.xlsx
+++ b/hhnk_threedi_tools/breaches/start_download_simulation/simulations_id.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\jacostabarragan\hhnk-threedi-tools\hhnk_threedi_tools\breaches\start_download_simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEE6690-18FA-4459-9174-E308568E5A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83DEDA11-B1C0-4334-B81B-7E1882BDD6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>scenario_name</t>
   </si>
@@ -41,6 +41,24 @@
   </si>
   <si>
     <t>SIZE_KB</t>
+  </si>
+  <si>
+    <t>date_simulation_created</t>
+  </si>
+  <si>
+    <t>date_simulation_downloaded</t>
+  </si>
+  <si>
+    <t>date_ldo_uploaded</t>
+  </si>
+  <si>
+    <t>schematitation_id</t>
+  </si>
+  <si>
+    <t>revision_number</t>
+  </si>
+  <si>
+    <t>model_id</t>
   </si>
 </sst>
 </file>
@@ -403,10 +421,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -414,18 +438,36 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>